<commit_message>
Fix lỗi cập nhật vi phạm
</commit_message>
<xml_diff>
--- a/report_vi_pham.xlsx
+++ b/report_vi_pham.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1253,6 +1253,66 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-30 14:05:42</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Không đội mũ bảo hiểm</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>evidence_images\violation_39_1769756742.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-30 14:05:44</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Không đội mũ bảo hiểm</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>evidence_images\violation_40_1769756744.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-30 14:05:50</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Không đội mũ bảo hiểm</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>evidence_images\violation_41_1769756750.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>